<commit_message>
feat: add references to the README.md file
</commit_message>
<xml_diff>
--- a/databases/test_01.xlsx
+++ b/databases/test_01.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,10 +458,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>19.0473724</v>
+        <v>19.0489792</v>
       </c>
       <c r="E2" t="n">
-        <v>-98.21006149999999</v>
+        <v>-98.21327170000001</v>
       </c>
     </row>
     <row r="3">
@@ -470,7 +470,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Avenida Reforma 100, Puebla, Puebla, Méxic</t>
+          <t>Paseo de la Reforma 222, Juárez, Cuauhtémoc, 06600 Ciudad de México, CDMX, México</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -479,10 +479,31 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>19.0683418</v>
+        <v>19.4287183</v>
       </c>
       <c r="E3" t="n">
-        <v>-98.2403383</v>
+        <v>-99.16129789999999</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ángel de la Independencia, Ciudad de México, México</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Empresa 03</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>19.4270032</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-99.16766819999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>